<commit_message>
edf-25 results with exact-round-trip handler and lr=1
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/edf/edf-25/edf-25_schedulables.xlsx
+++ b/workspace/framework_paper/edf/edf-25/edf-25_schedulables.xlsx
@@ -693,10 +693,10 @@
         <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -710,7 +710,7 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>